<commit_message>
Task 6: Replace the 1.5C budget with GCB 2025 170/525/1055 GtCO2.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Data_Inputs.xlsx
+++ b/Inputs/Canada_LNG_Data_Inputs.xlsx
@@ -1413,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2419,7 +2419,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -2433,99 +2433,117 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>IPCC AR6 WGIII Table SPM.2, remaining budget from 1 Jan 2020 for 50% chance of 1.5C</t>
+          <t>Global Carbon Budget 2025 (Friedlingstein et al., Earth Syst. Sci. Data). Remaining budget from the start of 2026, 50% likelihood. 1.5C.</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>https://www.ipcc.ch/report/ar6/wg3/</t>
+          <t>https://essd.copernicus.org/articles/18/3211/2026/</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2022 vintage</t>
+          <t>2025 (from 1 Jan 2026)</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>CO2 only, declines each year</t>
+          <t>Budget is CO2. Register emissions are GWP100 CO2e. The comparison is CO2e against a CO2 budget and is an approximation; a true CO2-only total is not derivable from this model.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>coal_plant_reference_mw</t>
+          <t>remaining_17c_budget</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>500</v>
+        <v>525</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MW</t>
+          <t>GtCO2</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>assumption</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>Comparator assumption</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>Not available</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr"/>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Global Carbon Budget 2025 (Friedlingstein et al., Earth Syst. Sci. Data). Remaining budget from the start of 2026, 50% likelihood. 1.7C.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://essd.copernicus.org/articles/18/3211/2026/</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2025 (from 1 Jan 2026)</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Budget is CO2. Register emissions are GWP100 CO2e. The comparison is CO2e against a CO2 budget and is an approximation; a true CO2-only total is not derivable from this model.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>coal_plant_capacity_factor</t>
+          <t>remaining_2c_budget</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.55</v>
+        <v>1055</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>fraction</t>
+          <t>GtCO2</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>assumption</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>Comparator assumption</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Not available</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr"/>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Global Carbon Budget 2025 (Friedlingstein et al., Earth Syst. Sci. Data). Remaining budget from the start of 2026, 50% likelihood. 2.0C.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://essd.copernicus.org/articles/18/3211/2026/</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2025 (from 1 Jan 2026)</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Budget is CO2. Register emissions are GWP100 CO2e. The comparison is CO2e against a CO2 budget and is an approximation; a true CO2-only total is not derivable from this model.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>coal_tco2e_per_mwh</t>
+          <t>coal_plant_reference_mw</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.95</v>
+        <v>500</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>tCO2e/MWh</t>
+          <t>MW</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2548,35 +2566,30 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>tmx_total_system_bpd</t>
+          <t>coal_plant_capacity_factor</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>890000</v>
+        <v>0.55</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>barrels per day</t>
+          <t>fraction</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>assumption</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Trans Mountain system capacity after the May 2024 expansion</t>
+          <t>Comparator assumption</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>https://www.transmountain.com/</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>2024</t>
+          <t>Not available</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
@@ -2584,15 +2597,15 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>lng_canada_ph1_year_1_utilisation</t>
+          <t>coal_tco2e_per_mwh</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.25</v>
+        <v>0.95</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>fraction</t>
+          <t>tCO2e/MWh</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2602,73 +2615,60 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Project-specific ramp for LNG Canada Phase 1, the only Canadian export terminal in operation. Informed by its actual startup: first cargo June 2025, Train 2 producing from November 2025. LNG Canada does not publish utilisation figures, so this is a judgement anchored on observed timing rather than a cited rate.</t>
+          <t>Comparator assumption</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>https://www.lngcanada.ca/</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>Replaces year_1_utilisation for this project only</t>
-        </is>
-      </c>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>lng_canada_ph1_year_2_utilisation</t>
+          <t>tmx_total_system_bpd</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.6</v>
+        <v>890000</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>fraction</t>
+          <t>barrels per day</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>cited</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Second year of the LNG Canada Phase 1 ramp. Judgement, anchored on the observed startup sequence.</t>
+          <t>Trans Mountain system capacity after the May 2024 expansion</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>https://www.lngcanada.ca/</t>
+          <t>https://www.transmountain.com/</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>Replaces year_2_utilisation for this project only</t>
-        </is>
-      </c>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>lng_canada_ph1_steady_state_utilisation</t>
+          <t>lng_canada_ph1_year_1_utilisation</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.85</v>
+        <v>0.25</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -2682,7 +2682,7 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Steady state for LNG Canada Phase 1, slightly above the 83.9 per cent global average. Judgement, not a published figure.</t>
+          <t>Project-specific ramp for LNG Canada Phase 1, the only Canadian export terminal in operation. Informed by its actual startup: first cargo June 2025, Train 2 producing from November 2025. LNG Canada does not publish utilisation figures, so this is a judgement anchored on observed timing rather than a cited rate.</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -2697,24 +2697,22 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Replaces steady_state_utilisation for this project only</t>
+          <t>Replaces year_1_utilisation for this project only</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>liquefaction_drive_default</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>gas_turbine</t>
-        </is>
+          <t>lng_canada_ph1_year_2_utilisation</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0.6</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>fraction</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2724,28 +2722,33 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Fallback drive type where a facility does not publish one. Applies only to small domestic and bunkering plants totalling 1.22 mtpa, several predating 2000. The choice between gas turbine and electric moves the total by under 0.2 MtCO2e a year.</t>
+          <t>Second year of the LNG Canada Phase 1 ramp. Judgement, anchored on the observed startup sequence.</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>https://www.lngcanada.ca/</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Fallback only for domestic plants that still carry not_published. Export and bunkering assets are recorded as gas_turbine. Electric drive is not assumed for any terminal.</t>
+          <t>Replaces year_2_utilisation for this project only</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>saint_john_utilisation</t>
+          <t>lng_canada_ph1_steady_state_utilisation</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.025</v>
+        <v>0.85</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -2754,52 +2757,54 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>assumption</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Actual throughput at the Saint John import terminal. Repsol's annual report records 8 TBtu regasified in 2023 and 10 TBtu in 2022, against 7.5 mtpa of nameplate capacity. Corroborated by the CER, which found the terminal at 4 per cent of send-out capacity in 2017, with cargo counts falling from 42 in 2011 to 5 in 2017.</t>
+          <t>Steady state for LNG Canada Phase 1, slightly above the 83.9 per cent global average. Judgement, not a published figure.</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>https://lngprime.com/americas/repsols-saint-john-lng-terminal-to-get-galileos-reliquefaction-tech/115035/</t>
+          <t>https://www.lngcanada.ca/</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Applying nameplate utilisation here overstates the terminal's emissions roughly thirtyfold</t>
+          <t>Replaces steady_state_utilisation for this project only</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>lng_energy_content</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>52</v>
+          <t>liquefaction_drive_default</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>gas_turbine</t>
+        </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MMBtu per tonne</t>
+          <t>category</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>method constant</t>
+          <t>assumption</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Energy content of LNG, used to convert reported throughput in energy units into tonnes.</t>
+          <t>Fallback drive type where a facility does not publish one. Applies only to small domestic and bunkering plants totalling 1.22 mtpa, several predating 2000. The choice between gas turbine and electric moves the total by under 0.2 MtCO2e a year.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -2809,22 +2814,22 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Also required for the per-kWh energy source comparison</t>
+          <t>Fallback only for domestic plants that still carry not_published. Export and bunkering assets are recorded as gas_turbine. Electric drive is not assumed for any terminal.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>lng_export_licence_max_term</t>
+          <t>saint_john_utilisation</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>50</v>
+        <v>0.025</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>fraction</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2834,193 +2839,188 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Maximum duration of an LNG export licence under the Canadian Energy Regulator Act, raised from 40 years by Bill C-15, Division 41 of Part 5, royal assent 26 March 2026. No 50 year licence has yet been issued: Cedar's licence, approved January 2026, is for 40 years. Precedent suggests holders will apply to extend, as they did when the ceiling rose from 25 to 40 in 2015.</t>
+          <t>Actual throughput at the Saint John import terminal. Repsol's annual report records 8 TBtu regasified in 2023 and 10 TBtu in 2022, against 7.5 mtpa of nameplate capacity. Corroborated by the CER, which found the terminal at 4 per cent of send-out capacity in 2017, with cargo counts falling from 42 in 2011 to 5 in 2017.</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>https://www.parl.ca/documentviewer/en/45-1/bill/C-15/royal-assent</t>
+          <t>https://lngprime.com/americas/repsols-saint-john-lng-terminal-to-get-galileos-reliquefaction-tech/115035/</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Gives the 50 year lifespan sensitivity a legal basis</t>
+          <t>Applying nameplate utilisation here overstates the terminal's emissions roughly thirtyfold</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>canada_2030_overshoot_gap</t>
+          <t>lng_energy_content</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>200</v>
+        <v>52</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MtCO2e</t>
+          <t>MMBtu per tonne</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>method constant</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Difference between projected 2030 emissions of about 646 MtCO2e and the legislated target range of 417 to 455. Expressing a figure as a share of this gap is harder to dismiss than expressing it as a share of an allowance that is not expected to be met.</t>
+          <t>Energy content of LNG, used to convert reported throughput in energy units into tonnes.</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>https://climateactiontracker.org/countries/canada/</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr"/>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>Also required for the per-kWh energy source comparison</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>upstream_ch4_share</t>
+          <t>lng_export_licence_max_term</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.3</v>
+        <v>50</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>fraction</t>
+          <t>years</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>cited</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Share of upstream oil and gas emissions that is methane rather than carbon dioxide. Required to apply the measurement correction and the GWP20 uplift to the methane portion only. Canada's 2023 National Inventory Report gives 20 per cent for the oil and gas sector nationally, but that includes oil sands, which are far more carbon dioxide intensive than gas production. British Columbia is gas-dominated, which raises the share, while its 51 per cent methane reduction by 2023 lowers it.</t>
+          <t>Maximum duration of an LNG export licence under the Canadian Energy Regulator Act, raised from 40 years by Bill C-15, Division 41 of Part 5, royal assent 26 March 2026. No 50 year licence has yet been issued: Cedar's licence, approved January 2026, is for 40 years. Precedent suggests holders will apply to extend, as they did when the ceiling rose from 25 to 40 in 2015.</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>https://gazette.gc.ca/rp-pr/p1/2023/2023-12-16/html/reg3-eng.html</t>
+          <t>https://www.parl.ca/documentviewer/en/45-1/bill/C-15/royal-assent</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Tested across 20 to 40 per cent</t>
+          <t>Gives the 50 year lifespan sensitivity a legal basis</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>upstream_measurement_correction</t>
+          <t>canada_2030_overshoot_gap</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1.5</v>
+        <v>200</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>multiplier</t>
+          <t>MtCO2e</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Factor by which peer-reviewed measurement studies find Canadian inventories understate upstream oil and gas methane. Three independent studies agree: 6,650 site measurements across Canada, an Alberta measurement-based inventory, and a British Columbia aircraft survey giving 1.7.</t>
+          <t>Difference between projected 2030 emissions of about 646 MtCO2e and the legislated target range of 417 to 455. Expressing a figure as a share of this gap is harder to dismiss than expressing it as a share of an allowance that is not expected to be met.</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41598-021-87610-3</t>
+          <t>https://climateactiontracker.org/countries/canada/</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2021</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr">
-        <is>
-          <t>Applied to the methane portion only</t>
-        </is>
-      </c>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>liquefaction_gas_turbine</t>
+          <t>upstream_ch4_share</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>tCO2e per t LNG</t>
+          <t>fraction</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>assumption</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Liquefaction intensity for gas turbine drive, implied by LNG Canada's environmental assessment of roughly 4 MtCO2e per year against 14 mtpa of capacity.</t>
+          <t>Share of upstream oil and gas emissions that is methane rather than carbon dioxide. Required to apply the measurement correction and the GWP20 uplift to the methane portion only. Canada's 2023 National Inventory Report gives 20 per cent for the oil and gas sector nationally, but that includes oil sands, which are far more carbon dioxide intensive than gas production. British Columbia is gas-dominated, which raises the share, while its 51 per cent methane reduction by 2023 lowers it.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>https://www.projects.eao.gov.bc.ca/p/lng-canada-export-terminal</t>
+          <t>https://gazette.gc.ca/rp-pr/p1/2023/2023-12-16/html/reg3-eng.html</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Equals Emission Factors liquefaction central. Applied to every terminal for its whole operating life as of August 2026.</t>
+          <t>Tested across 20 to 40 per cent</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>liquefaction_electric</t>
+          <t>upstream_measurement_correction</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.12</v>
+        <v>1.5</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>tCO2e per t LNG</t>
+          <t>multiplier</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3030,28 +3030,33 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Liquefaction intensity for electric drive. Pembina Institute electrified LNG scenario. Woodfibre claims 0.059 for its own facility.</t>
+          <t>Factor by which peer-reviewed measurement studies find Canadian inventories understate upstream oil and gas methane. Three independent studies agree: 6,650 site measurements across Canada, an Alberta measurement-based inventory, and a British Columbia aircraft survey giving 1.7.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>https://www.pembina.org/</t>
+          <t>https://www.nature.com/articles/s41598-021-87610-3</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2021</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>Retained for reference. Not used in the central case. Matches Emission Factors range_low; applies only if electrification is contracted and delivered.</t>
+          <t>Applied to the methane portion only</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>bc_lng_emission_intensity_benchmark</t>
+          <t>liquefaction_gas_turbine</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.16</v>
+        <v>0.29</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -3060,42 +3065,42 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Legislated benchmark under British Columbia's Greenhouse Gas Industrial Reporting and Control Act, covering gas entering the facility to loading onto ships. Facilities above it must buy offsets, buy permits from a better-performing facility, or pay into a technology fund.</t>
+          <t>Liquefaction intensity for gas turbine drive, implied by LNG Canada's environmental assessment of roughly 4 MtCO2e per year against 14 mtpa of capacity.</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>https://www2.gov.bc.ca/gov/content/environment/climate-change/industry/reporting</t>
+          <t>https://www.projects.eao.gov.bc.ca/p/lng-canada-export-terminal</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>A gas turbine facility at 0.29 exceeds this by 0.13, about 1.8 Mt/yr across 14 mtpa</t>
+          <t>Equals Emission Factors liquefaction central. Applied to every terminal for its whole operating life as of August 2026.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>route_bc_to_northeast_asia_nm</t>
+          <t>liquefaction_electric</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3800</v>
+        <v>0.12</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>nautical miles</t>
+          <t>tCO2e per t LNG</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3105,37 +3110,32 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Oxford Institute for Energy Studies, west coast Canada to Tokyo, as cited by CAPP. Black &amp; Veatch citing PortWorld gives approximately 4,000 nm for the same run.</t>
+          <t>Liquefaction intensity for electric drive. Pembina Institute electrified LNG scenario. Woodfibre claims 0.059 for its own facility.</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>https://www.capp.ca/wp-content/uploads/2026/05/The-Case-for-Canadian-LNG-April-17-2026.pdf</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>2026</t>
+          <t>https://www.pembina.org/</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>One way</t>
+          <t>Retained for reference. Not used in the central case. Matches Emission Factors range_low; applies only if electrification is contracted and delivered.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>route_us_gulf_to_northeast_asia_nm</t>
+          <t>bc_lng_emission_intensity_benchmark</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>9200</v>
+        <v>0.16</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>nautical miles</t>
+          <t>tCO2e per t LNG</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3145,32 +3145,37 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>US Gulf Coast to Tokyo via the Panama Canal. Reference point only, used to test the industry's proximity claim.</t>
+          <t>Legislated benchmark under British Columbia's Greenhouse Gas Industrial Reporting and Control Act, covering gas entering the facility to loading onto ships. Facilities above it must buy offsets, buy permits from a better-performing facility, or pay into a technology fund.</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>https://www.bv.com/en-US/perspectives/geographic-location-magnifies-advantages-for-north-american-lng-exports</t>
+          <t>https://www2.gov.bc.ca/gov/content/environment/climate-change/industry/reporting</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2016</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>One way</t>
+          <t>A gas turbine facility at 0.29 exceeds this by 0.13, about 1.8 Mt/yr across 14 mtpa</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>voyage_days_bc_to_north_asia</t>
+          <t>route_bc_to_northeast_asia_nm</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>10</v>
+        <v>3800</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>days</t>
+          <t>nautical miles</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3180,33 +3185,37 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Reported at the time of LNG Canada's first cargo, against 20 days from the US Gulf Coast via Panama.</t>
+          <t>Oxford Institute for Energy Studies, west coast Canada to Tokyo, as cited by CAPP. Black &amp; Veatch citing PortWorld gives approximately 4,000 nm for the same run.</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>https://www.theglobeandmail.com/business/article-lng-canada-liquefied-natural-gas-shipment-asia/</t>
+          <t>https://www.capp.ca/wp-content/uploads/2026/05/The-Case-for-Canadian-LNG-April-17-2026.pdf</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr"/>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>One way</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ocean_transport_intensity_range_low</t>
+          <t>route_us_gulf_to_northeast_asia_nm</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.05</v>
+        <v>9200</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>tCO2e per t LNG delivered</t>
+          <t>nautical miles</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3216,33 +3225,32 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Peer reviewed supplier-specific LNG lifecycle assessment. Ocean transport ranges from 0.05 tCO2e/t (short routes) to 0.31 (long routes), a sixfold spread, confirming route matters.</t>
+          <t>US Gulf Coast to Tokyo via the Panama Canal. Reference point only, used to test the industry's proximity claim.</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>https://pubs.acs.org/doi/10.1021/acssuschemeng.1c03307</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr"/>
+          <t>https://www.bv.com/en-US/perspectives/geographic-location-magnifies-advantages-for-north-american-lng-exports</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>One way</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ocean_transport_intensity_range_high</t>
+          <t>voyage_days_bc_to_north_asia</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.31</v>
+        <v>10</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>tCO2e per t LNG delivered</t>
+          <t>days</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3252,17 +3260,17 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Same source. Upper end corresponds to long routes such as US Gulf Coast to Taiwan.</t>
+          <t>Reported at the time of LNG Canada's first cargo, against 20 days from the US Gulf Coast via Panama.</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>https://pubs.acs.org/doi/10.1021/acssuschemeng.1c03307</t>
+          <t>https://www.theglobeandmail.com/business/article-lng-canada-liquefied-natural-gas-shipment-asia/</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr"/>
@@ -3270,95 +3278,87 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>route_atlantic_routing_factor</t>
+          <t>ocean_transport_intensity_range_low</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1.125</v>
+        <v>0.05</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>multiplier</t>
+          <t>tCO2e per t LNG delivered</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>cited</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Ratio of actual sailing distance to great circle distance for a North Atlantic crossing. Calibrated on Saint John NB to Rotterdam: SeaRates gives 5,648 km (3,050 nm) against a great circle of 2,712 nm. Applied to Atlantic routes only.</t>
+          <t>Peer reviewed supplier-specific LNG lifecycle assessment. Ocean transport ranges from 0.05 tCO2e/t (short routes) to 0.31 (long routes), a sixfold spread, confirming route matters.</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>https://www.searates.com/distance-time/</t>
+          <t>https://pubs.acs.org/doi/10.1021/acssuschemeng.1c03307</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>Not applied to Pacific routes</t>
-        </is>
-      </c>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>route_baie_comeau_to_rotterdam_nm</t>
+          <t>ocean_transport_intensity_range_high</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2980</v>
+        <v>0.31</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>nautical miles</t>
+          <t>tCO2e per t LNG delivered</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>cited</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Great circle from port coordinates, scaled by the Atlantic routing factor.</t>
+          <t>Same source. Upper end corresponds to long routes such as US Gulf Coast to Taiwan.</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>https://www.searates.com/distance-time/</t>
+          <t>https://pubs.acs.org/doi/10.1021/acssuschemeng.1c03307</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H53" s="4" t="inlineStr">
-        <is>
-          <t>Estimate, not a published sailing distance</t>
-        </is>
-      </c>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>route_fermeuse_to_rotterdam_nm</t>
+          <t>route_atlantic_routing_factor</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2470</v>
+        <v>1.125</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>nautical miles</t>
+          <t>multiplier</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Great circle from port coordinates, scaled by the Atlantic routing factor.</t>
+          <t>Ratio of actual sailing distance to great circle distance for a North Atlantic crossing. Calibrated on Saint John NB to Rotterdam: SeaRates gives 5,648 km (3,050 nm) against a great circle of 2,712 nm. Applied to Atlantic routes only.</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
@@ -3383,18 +3383,18 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>Estimate, not a published sailing distance</t>
+          <t>Not applied to Pacific routes</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>route_saint_john_to_rotterdam_nm</t>
+          <t>route_baie_comeau_to_rotterdam_nm</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>3050</v>
+        <v>2980</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -3403,12 +3403,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>Actual sailing distance, 5,648 km, from the SeaRates port-to-port calculator.</t>
+          <t>Great circle from port coordinates, scaled by the Atlantic routing factor.</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -3423,62 +3423,62 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>The calibration point for the Atlantic routing factor</t>
+          <t>Estimate, not a published sailing distance</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>lng_carrier_aer_gco2_per_dwt_nm</t>
+          <t>route_fermeuse_to_rotterdam_nm</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>8.5</v>
+        <v>2470</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>gCO2 per DWT per nautical mile</t>
+          <t>nautical miles</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>IMO Data Collection System 2023 annual report, LNG carrier fleet average Annual Efficiency Ratio, as reported in an analysis of EU MRV 2023 data. Annual figure, so it already includes ballast legs.</t>
+          <t>Great circle from port coordinates, scaled by the Atlantic routing factor.</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>https://www.mdpi.com/2077-1312/13/8/1437</t>
+          <t>https://www.searates.com/distance-time/</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>Use to scale shipping by route distance</t>
+          <t>Estimate, not a published sailing distance</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>lng_carrier_kgco2_per_nm</t>
+          <t>route_saint_john_to_rotterdam_nm</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>940</v>
+        <v>3050</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>kg CO2 per nautical mile</t>
+          <t>nautical miles</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3488,112 +3488,117 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>EU JRC analysis of 2019 EU MRV data. LNG carriers are the highest-emitting ship category per nautical mile travelled.</t>
+          <t>Actual sailing distance, 5,648 km, from the SeaRates port-to-port calculator.</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>https://publications.jrc.ec.europa.eu/repository/bitstream/JRC128870/JRC128870_01.pdf</t>
+          <t>https://www.searates.com/distance-time/</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>Per ship, not per tonne of cargo</t>
+          <t>The calibration point for the Atlantic routing factor</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>lng_carrier_methane_slip_uplift</t>
+          <t>lng_carrier_aer_gco2_per_dwt_nm</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1.44</v>
+        <v>8.5</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>multiplier</t>
+          <t>gCO2 per DWT per nautical mile</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>cited</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>Derived from the first primary measurement study of an LNG carrier voyage, which recorded 68.1 t CH4 against 4,600 t CO2. At GWP100 of 29.8 this raises voyage emissions by about 44 per cent. Methane slip averaged 3.8 per cent across engines.</t>
+          <t>IMO Data Collection System 2023 annual report, LNG carrier fleet average Annual Efficiency Ratio, as reported in an analysis of EU MRV 2023 data. Annual figure, so it already includes ballast legs.</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>https://pubs.acs.org/doi/10.1021/acs.est.2c01383</t>
+          <t>https://www.mdpi.com/2077-1312/13/8/1437</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t>Applies to the shipping stage only</t>
+          <t>Use to scale shipping by route distance</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>cargo_tonnes_per_dwt</t>
+          <t>lng_carrier_kgco2_per_nm</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.85</v>
+        <v>940</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>fraction</t>
+          <t>kg CO2 per nautical mile</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>cited</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>Model assumption - typical ratio of LNG cargo tonnes to carrier deadweight. Needed to convert AER, which is per DWT, into emissions per tonne of cargo.</t>
+          <t>EU JRC analysis of 2019 EU MRV data. LNG carriers are the highest-emitting ship category per nautical mile travelled.</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>https://publications.jrc.ec.europa.eu/repository/bitstream/JRC128870/JRC128870_01.pdf</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2019</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>Sensitivity worth testing</t>
+          <t>Per ship, not per tonne of cargo</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>tmx_oil_lifecycle_per_barrel</t>
+          <t>lng_carrier_methane_slip_uplift</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.513</v>
+        <v>1.44</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>tCO2e/bbl</t>
+          <t>multiplier</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3603,53 +3608,128 @@
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>Sum of upstream 0.075, transport 0.008 and combustion 0.43</t>
+          <t>Derived from the first primary measurement study of an LNG carrier voyage, which recorded 68.1 t CH4 against 4,600 t CO2. At GWP100 of 29.8 this raises voyage emissions by about 44 per cent. Methane slip averaged 3.8 per cent across engines.</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Not available</t>
-        </is>
-      </c>
-      <c r="H60" s="4" t="inlineStr"/>
+          <t>https://pubs.acs.org/doi/10.1021/acs.est.2c01383</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>Applies to the shipping stage only</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>cargo_tonnes_per_dwt</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>Model assumption - typical ratio of LNG cargo tonnes to carrier deadweight. Needed to convert AER, which is per DWT, into emissions per tonne of cargo.</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>Sensitivity worth testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>tmx_oil_lifecycle_per_barrel</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>0.513</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>tCO2e/bbl</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>Sum of upstream 0.075, transport 0.008 and combustion 0.43</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>liquefaction_electrification_assumed</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Model assumption - no external source</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>Not available</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
+      <c r="G63" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="H63" t="inlineStr">
         <is>
           <t>Electric drive is not assumed for any terminal. Of the projects claiming electrification, only Cedar and Woodfibre have interconnection works under construction; the remainder rest on memoranda of understanding, aspirations conditional on transmission that has not been built, or statements with no firm date. Ksi Lisims holds an MOU with BC Hydro for up to 600 MW conditional on the North Coast Transmission Line expansion, which is not built. LNG Canada Phase 2 states an intention to transition to electric motors as more renewable power becomes available, with no date and no contracted supply. There is not sufficient evidence that electric drive will be in use at these facilities, and a commitment contingent on infrastructure that does not exist is not a basis for lowering the emissions factor. Where electrification is later contracted and built, this assumption should be revisited.</t>
         </is>

</xml_diff>

<commit_message>
Task 2: Move placeholder start year onto the Parameters sheet and report 2030/2033/2035.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Data_Inputs.xlsx
+++ b/Inputs/Canada_LNG_Data_Inputs.xlsx
@@ -1413,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3732,6 +3732,44 @@
       <c r="H63" t="inlineStr">
         <is>
           <t>Electric drive is not assumed for any terminal. Of the projects claiming electrification, only Cedar and Woodfibre have interconnection works under construction; the remainder rest on memoranda of understanding, aspirations conditional on transmission that has not been built, or statements with no firm date. Ksi Lisims holds an MOU with BC Hydro for up to 600 MW conditional on the North Coast Transmission Line expansion, which is not built. LNG Canada Phase 2 states an intention to transition to electric motors as more renewable power becomes available, with no date and no contracted supply. There is not sufficient evidence that electric drive will be in use at these facilities, and a commitment contingent on infrastructure that does not exist is not a basis for lowering the emissions factor. Where electrification is later contracted and built, this assumption should be revisited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>assumed_first_export_year_if_missing</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>2030</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Named model parameter: calendar start year filled when Asset Register first_export_year is blank. In-scope assets: tilbury_phase_2, marinvest_baie_comeau, summit_lake_pg_lng, fermeuse_energy_flng, discovery_t1t4, kanata_lng. With licence-end stops, every dated authorised end year is 2056-2066; the published panel tail is entirely this placeholder.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Central value 2030. Sensitivity at 2033 and 2035 is reported. Summit Lake states a 30-year life; the other five use lifecycle_years_default.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Task 3: Decouple Monte Carlo: sample physics, apply ECCC prices after.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Data_Inputs.xlsx
+++ b/Inputs/Canada_LNG_Data_Inputs.xlsx
@@ -1413,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3770,6 +3770,82 @@
       <c r="H64" t="inlineStr">
         <is>
           <t>Central value 2030. Sensitivity at 2033 and 2035 is reported. Summit Lake states a 30-year life; the other five use lifecycle_years_default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>monte_carlo_seed</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>20260828</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Seed for the decoupled physics Monte Carlo (numpy Generator). Recorded in the run manifest.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Do not reuse a draw sequence across published runs without recording a new seed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>monte_carlo_n_draws</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Number of physics draws. Price schedules are applied after, not rebuilt inside the loop.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>10,000 draws for stable 5th/95th percentiles.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Task 4: Tie documented territorial shares to the computed 18.5/5.6/75.9 split.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Data_Inputs.xlsx
+++ b/Inputs/Canada_LNG_Data_Inputs.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Across all Canadian LNG assets, about 16 per cent of emissions are Canada territorial, 5 per cent are international bunkers, and 80 per cent are foreign territorial. LNG carrier shipping is itself an international bunker, so it lands nowhere.</t>
+          <t>Across all Canadian LNG assets, 18.5 per cent of emissions are Canada territorial, 5.6 per cent are international bunkers, and 75.9 per cent are foreign territorial. LNG carrier shipping is itself an international bunker, so it lands nowhere. These shares are the life-average split; the model asserts them every run.</t>
         </is>
       </c>
     </row>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="P2" s="4" t="inlineStr">
         <is>
-          <t>Only about 16 per cent of these emissions land on Canada's inventory. The rest is counted by the importing country or by nobody.</t>
+          <t>18 per cent of export-chain emissions land on Canada's inventory, 3 per cent are international bunkers, and 79 per cent are foreign territorial (importing-country inventory).</t>
         </is>
       </c>
     </row>
@@ -4549,7 +4549,7 @@
       </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>Under UNFCCC accounting international bunkers are reported separately and attributed to no country. Roughly 80 per cent of this chain's emissions land nowhere.</t>
+          <t>Under UNFCCC accounting international bunkers are reported separately and attributed to no country. 81 per cent of this chain's emissions are bunkers (land nowhere); the remaining 19 per cent is Canada territorial (upstream, pipeline, liquefaction).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Task B: Narrow headline results to export-chain assets via named Parameters-sheet scope filter. Lifetime 9558.2 to 9315.3 Mt; peak 309.1 to 298.7 Mt in 2037; ECCC 4267 to 4164 CAD bn. Eight non-export assets (242.9 Mt) stay in the register. Liquefaction remains 0.29. Locked assertions left at the old values for Task C.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Data_Inputs.xlsx
+++ b/Inputs/Canada_LNG_Data_Inputs.xlsx
@@ -1413,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3846,6 +3846,86 @@
       <c r="H66" t="inlineStr">
         <is>
           <t>10,000 draws for stable 5th/95th percentiles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>headline_scope_chains</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>export</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>comma-separated chains</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Model assumption - no external source</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Headline results include assets whose chain is in headline_scope_chains and whose calc_group is in headline_scope_calc_groups. Domestic peak-shaving and other non-export assets are out of headline; they stay in the register. Inventing a 1971/1976 retirement date is not supported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>headline_scope_calc_groups</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>operating,under_construction,proposed</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>comma-separated calc_groups</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Model assumption - no external source</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Headline results include assets whose chain is in headline_scope_chains and whose calc_group is in headline_scope_calc_groups. Domestic peak-shaving and other non-export assets are out of headline; they stay in the register. Inventing a 1971/1976 retirement date is not supported.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Task C: Re-lock headline assertions after the export-scope change (lifetime 9558.2 to 9315.3; peak 309.1 to 298.7 in 2037; territorial 18.5/5.6/75.9 to 18.0/3.4/78.6). Update README, Chains applies_to, and Data Inputs README. Deliberate scope change, not a silent correction.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Data_Inputs.xlsx
+++ b/Inputs/Canada_LNG_Data_Inputs.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Across all Canadian LNG assets, 18.5 per cent of emissions are Canada territorial, 5.6 per cent are international bunkers, and 75.9 per cent are foreign territorial. LNG carrier shipping is itself an international bunker, so it lands nowhere. These shares are the life-average split; the model asserts them every run.</t>
+          <t>Across the export-chain headline (headline_scope_chains=export; headline_scope_calc_groups=operating,under_construction,proposed), 18.0 per cent of emissions are Canada territorial, 3.4 per cent are international bunkers, and 78.6 per cent are foreign territorial. LNG carrier shipping is itself an international bunker, so it lands nowhere. These shares are the life-average split; the model asserts them every run. Eight non-export assets totalling 242.9 MtCO2e stay in the register.</t>
         </is>
       </c>
     </row>
@@ -4552,7 +4552,7 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>45.4 mtpa active, 12.7 mtpa early stage</t>
+          <t>100.1 mtpa (14.0 operating, 5.4 under construction, 80.7 proposed)</t>
         </is>
       </c>
       <c r="P2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Correct regasification citation from Gan et al. (2024) to Mukherjee et al. (2025).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Data_Inputs.xlsx
+++ b/Inputs/Canada_LNG_Data_Inputs.xlsx
@@ -1360,12 +1360,12 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>0.021 tCO2e per t LNG. Gan et al. (2024), Communications Earth &amp; Environment, https://doi.org/10.1038/s43247-024-01988-2 : peer-reviewed US LNG lifecycle assessment placing regasification at 0.021 tCO2e/t. Adopted 3 September 2026, replacing an uncited 0.04 that sat above the top of the IEA range below. The previous 0.04 was labelled RMI Oil Climate Index; no OCI+ table or page states 0.04 t/t.</t>
+          <t>0.021 tCO2e per t LNG. Mukherjee et al. (2025), Communications Earth &amp; Environment 6:16, https://doi.org/10.1038/s43247-024-01988-2 : peer-reviewed US LNG lifecycle assessment placing regasification at 0.021 tCO2e/t. Adopted 3 September 2026, replacing an uncited 0.04 that sat above the top of the IEA range below. The previous 0.04 was labelled RMI Oil Climate Index; no OCI+ table or page states 0.04 t/t.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>IEA (2025), Assessing Emissions from LNG Supply and Abatement Options, IEA, Paris, CC BY 4.0, page 16: "Total GHG emissions from regasification are around 0.2-0.5 g CO2-eq/MJ of gas regasified." https://iea.blob.core.windows.net/assets/df9b1bed-4e16-4db8-bec5-a5fa117a9130/AssessingemissionsfromLNGsupplyandabatementoptions.pdf . Converted at the report's own stated basis of 55 MJ per kg of methane (footnote 2, page 7): 0.2 g/MJ = 0.011 and 0.5 g/MJ = 0.0275 tCO2e per tonne. IEA takes 1 t methane as 30 t CO2 on a 100-year GWP, against this model's 29.8. The Gan et al. central of 0.021 sits inside this range.</t>
+          <t>IEA (2025), Assessing Emissions from LNG Supply and Abatement Options, IEA, Paris, CC BY 4.0, page 16: "Total GHG emissions from regasification are around 0.2-0.5 g CO2-eq/MJ of gas regasified." https://iea.blob.core.windows.net/assets/df9b1bed-4e16-4db8-bec5-a5fa117a9130/AssessingemissionsfromLNGsupplyandabatementoptions.pdf . Converted at the report's own stated basis of 55 MJ per kg of methane (footnote 2, page 7): 0.2 g/MJ = 0.011 and 0.5 g/MJ = 0.0275 tCO2e per tonne. IEA takes 1 t methane as 30 t CO2 on a 100-year GWP, against this model's 29.8. The Mukherjee et al. central of 0.021 sits inside this range.</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">

</xml_diff>